<commit_message>
update format excel test cases deep audit
</commit_message>
<xml_diff>
--- a/docs/qc/testcases/UC-EXBOT-deep-audit/UC-EXBOT-deep-audit_testcases_v1.xlsx
+++ b/docs/qc/testcases/UC-EXBOT-deep-audit/UC-EXBOT-deep-audit_testcases_v1.xlsx
@@ -268,7 +268,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -512,11 +512,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -802,6 +808,36 @@
     <xf numFmtId="166" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -895,104 +931,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0"/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>2</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3019425" cy="6562725"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="image3.png" title="Image"/>
-        <cNvPicPr preferRelativeResize="0"/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0"/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>9</col>
-      <colOff>0</colOff>
-      <row>2</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3048000" cy="6553200"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="image4.png" title="Image"/>
-        <cNvPicPr preferRelativeResize="0"/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0"/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>11</col>
-      <colOff>923925</colOff>
-      <row>1</row>
-      <rowOff>180975</rowOff>
-    </from>
-    <ext cx="3009900" cy="6562725"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="image2.png" title="Image"/>
-        <cNvPicPr preferRelativeResize="0"/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1694,7 +1632,11 @@
           <t>Project Code:</t>
         </is>
       </c>
-      <c r="E18" s="93" t="n"/>
+      <c r="E18" s="93" t="inlineStr">
+        <is>
+          <t>BNZA-Exbot</t>
+        </is>
+      </c>
       <c r="H18" s="5" t="n"/>
       <c r="I18" s="92" t="inlineStr">
         <is>
@@ -1724,7 +1666,11 @@
           <t>Document Code:</t>
         </is>
       </c>
-      <c r="E19" s="94" t="n"/>
+      <c r="E19" s="94" t="inlineStr">
+        <is>
+          <t>UC Deep Audit</t>
+        </is>
+      </c>
       <c r="H19" s="5" t="n"/>
       <c r="I19" s="92" t="inlineStr">
         <is>
@@ -1754,7 +1700,11 @@
           <t>Created By:</t>
         </is>
       </c>
-      <c r="E20" s="94" t="n"/>
+      <c r="E20" s="94" t="inlineStr">
+        <is>
+          <t>Linh.Mai</t>
+        </is>
+      </c>
       <c r="H20" s="5" t="n"/>
       <c r="I20" s="92" t="inlineStr">
         <is>
@@ -1822,7 +1772,11 @@
           <t>Created Date:</t>
         </is>
       </c>
-      <c r="E22" s="95" t="n"/>
+      <c r="E22" s="95" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
       <c r="H22" s="5" t="n"/>
       <c r="I22" s="92" t="inlineStr">
         <is>
@@ -1856,7 +1810,11 @@
           <t>Version</t>
         </is>
       </c>
-      <c r="E23" s="96" t="n"/>
+      <c r="E23" s="96" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
       <c r="H23" s="5" t="n"/>
       <c r="I23" s="92" t="inlineStr">
         <is>
@@ -8348,43 +8306,43 @@
       <c r="Y1" s="7" t="n"/>
       <c r="Z1" s="7" t="n"/>
     </row>
-    <row r="2" ht="23.25" customHeight="1" s="85">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2" ht="20" customHeight="1" s="85">
+      <c r="A2" s="109" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="109" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="110" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="110" t="inlineStr">
         <is>
           <t>Contents of update</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="110" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="110" t="inlineStr">
         <is>
           <t>Created By/Updated By</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="110" t="inlineStr">
         <is>
           <t>Reviewer</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="H2" s="110" t="inlineStr">
         <is>
           <t>Approver</t>
         </is>
@@ -8408,36 +8366,37 @@
       <c r="Y2" s="12" t="n"/>
       <c r="Z2" s="12" t="n"/>
     </row>
-    <row r="3" ht="17.25" customHeight="1" s="85">
-      <c r="A3" s="13" t="n">
+    <row r="3" ht="20" customHeight="1" s="85">
+      <c r="A3" s="111" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="14">
-        <f>Cover!E22</f>
-        <v/>
+      <c r="B3" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
       </c>
-      <c r="C3" s="15" t="inlineStr">
+      <c r="C3" s="113" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="111" t="inlineStr">
         <is>
           <t>Create New</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="111" t="inlineStr">
         <is>
           <t>Create New</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F3" s="114" t="inlineStr">
         <is>
-          <t>lien.le</t>
+          <t>Linh.Mai</t>
         </is>
       </c>
-      <c r="G3" s="18" t="n"/>
-      <c r="H3" s="19" t="n"/>
+      <c r="G3" s="114" t="inlineStr"/>
+      <c r="H3" s="114" t="inlineStr"/>
       <c r="I3" s="20" t="n"/>
       <c r="J3" s="20" t="n"/>
       <c r="K3" s="20" t="n"/>
@@ -15339,1063 +15298,1084 @@
   <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="17.8984375" customWidth="1" style="75" min="1" max="1"/>
-    <col width="23.69921875" customWidth="1" style="75" min="2" max="3"/>
-    <col width="37.5" customWidth="1" style="75" min="4" max="4"/>
-    <col width="20.19921875" customWidth="1" style="75" min="5" max="5"/>
-    <col width="24.19921875" customWidth="1" style="75" min="6" max="6"/>
+    <col width="8" customWidth="1" style="75" min="1" max="1"/>
+    <col width="80" customWidth="1" style="75" min="2" max="3"/>
+    <col width="80" customWidth="1" style="85" min="3" max="3"/>
+    <col width="80" customWidth="1" style="75" min="4" max="4"/>
+    <col width="80" customWidth="1" style="75" min="5" max="5"/>
+    <col width="10" customWidth="1" style="75" min="6" max="6"/>
     <col width="12.59765625" customWidth="1" style="75" min="7" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.4" customHeight="1" s="85">
-      <c r="A1" s="67" t="inlineStr">
+    <row r="1" ht="27" customHeight="1" s="85">
+      <c r="A1" s="105" t="inlineStr">
         <is>
           <t>TC ID</t>
         </is>
       </c>
-      <c r="B1" s="67" t="inlineStr">
+      <c r="B1" s="105" t="inlineStr">
         <is>
           <t>Test Title/Summary of test cases</t>
         </is>
       </c>
-      <c r="C1" s="68" t="inlineStr">
+      <c r="C1" s="106" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="D1" s="67" t="inlineStr">
+      <c r="D1" s="105" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="E1" s="67" t="inlineStr">
+      <c r="E1" s="105" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="67" t="inlineStr">
+      <c r="F1" s="105" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="85">
-      <c r="B2" s="99" t="inlineStr">
+    <row r="2" ht="27" customHeight="1" s="85">
+      <c r="A2" s="107" t="n"/>
+      <c r="B2" s="108" t="inlineStr">
         <is>
           <t>I. Operation: Periodic Deep Audit (deep-audit)</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" s="85">
-      <c r="B3" s="99" t="inlineStr">
+      <c r="C2" s="107" t="n"/>
+      <c r="D2" s="107" t="n"/>
+      <c r="E2" s="107" t="n"/>
+      <c r="F2" s="107" t="n"/>
+    </row>
+    <row r="3" ht="39" customHeight="1" s="85">
+      <c r="A3" s="107" t="n"/>
+      <c r="B3" s="108" t="inlineStr">
         <is>
           <t>I.1. Functional verification — Operation: Periodic Deep Audit (deep-audit)</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1" s="85">
-      <c r="A4" s="100" t="inlineStr">
+      <c r="C3" s="107" t="n"/>
+      <c r="D3" s="107" t="n"/>
+      <c r="E3" s="107" t="n"/>
+      <c r="F3" s="107" t="n"/>
+    </row>
+    <row r="4" ht="123" customHeight="1" s="85">
+      <c r="A4" s="107" t="inlineStr">
         <is>
           <t>TC_001</t>
         </is>
       </c>
-      <c r="B4" s="100" t="inlineStr">
+      <c r="B4" s="107" t="inlineStr">
         <is>
           <t>Verify the deep-audit happy path completes without triggering SAFE_MODE</t>
         </is>
       </c>
-      <c r="C4" s="100" t="inlineStr">
+      <c r="C4" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status with no hedge size mismatch. 2. No stuck markers are set (`stop_trigger_crossed_at` and `stop_replacing_started_at` are both NULL). 3. Hyperliquid API is reachable and returns valid clearinghouseState and marginSummary.</t>
         </is>
       </c>
-      <c r="D4" s="100" t="inlineStr">
+      <c r="D4" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit cron worker for the bot. 2. Let the worker read bot state from D1, call HL clearinghouseState (weight=2), verify short size matches `last_known_hl_short_size`, check stuck markers, fetch marginSummary, and update `last_audit_at`.</t>
         </is>
       </c>
-      <c r="E4" s="100" t="inlineStr">
+      <c r="E4" s="107" t="inlineStr">
         <is>
           <t>1. The audit completes successfully: `hedge_legs.margin_status` is updated from HL, `hedge_legs.last_audit_at` is set to the current timestamp, and `queue_idempotency` row is inserted with `state='succeeded'`. No SAFE_MODE entry occurs. (Reference: AC-DA-01, FR-EXBOT-016.)</t>
         </is>
       </c>
-      <c r="F4" s="100" t="inlineStr">
+      <c r="F4" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" s="85">
-      <c r="A5" s="100" t="inlineStr">
+    <row r="5" ht="63" customHeight="1" s="85">
+      <c r="A5" s="107" t="inlineStr">
         <is>
           <t>TC_002</t>
         </is>
       </c>
-      <c r="B5" s="100" t="inlineStr">
+      <c r="B5" s="107" t="inlineStr">
         <is>
           <t>Verify `last_audit_at` is updated after every successful deep-audit cycle</t>
         </is>
       </c>
-      <c r="C5" s="100" t="inlineStr">
+      <c r="C5" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. A previous deep-audit has set `hedge_legs.last_audit_at` to a known timestamp.</t>
         </is>
       </c>
-      <c r="D5" s="100" t="inlineStr">
+      <c r="D5" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit cron worker. 2. After the worker completes, read the `hedge_legs.last_audit_at` value.</t>
         </is>
       </c>
-      <c r="E5" s="100" t="inlineStr">
+      <c r="E5" s="107" t="inlineStr">
         <is>
           <t>1. `hedge_legs.last_audit_at` is updated to the current timestamp (later than the previous value). (Reference: FR-EXBOT-016, UC Step 7.)</t>
         </is>
       </c>
-      <c r="F5" s="100" t="inlineStr">
+      <c r="F5" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1" s="85">
-      <c r="A6" s="100" t="inlineStr">
+    <row r="6" ht="75" customHeight="1" s="85">
+      <c r="A6" s="107" t="inlineStr">
         <is>
           <t>TC_003</t>
         </is>
       </c>
-      <c r="B6" s="100" t="inlineStr">
+      <c r="B6" s="107" t="inlineStr">
         <is>
           <t>Verify margin status is updated from HL marginSummary after deep-audit</t>
         </is>
       </c>
-      <c r="C6" s="100" t="inlineStr">
+      <c r="C6" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status with an existing `hedge_legs.margin_status` value. 2. HL marginSummary returns a different margin status than the current D1 value.</t>
         </is>
       </c>
-      <c r="D6" s="100" t="inlineStr">
+      <c r="D6" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit cron worker. 2. After the worker completes, read the `hedge_legs.margin_status` value in D1.</t>
         </is>
       </c>
-      <c r="E6" s="100" t="inlineStr">
+      <c r="E6" s="107" t="inlineStr">
         <is>
           <t>1. `hedge_legs.margin_status` is updated to match the fresh HL marginSummary data. (Reference: FR-EXBOT-016, FR-EXBOT-060, UC Step 6.)</t>
         </is>
       </c>
-      <c r="F6" s="100" t="inlineStr">
+      <c r="F6" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1" s="85">
-      <c r="A7" s="100" t="inlineStr">
+    <row r="7" ht="99" customHeight="1" s="85">
+      <c r="A7" s="107" t="inlineStr">
         <is>
           <t>TC_004</t>
         </is>
       </c>
-      <c r="B7" s="100" t="inlineStr">
+      <c r="B7" s="107" t="inlineStr">
         <is>
           <t>Verify deep-audit processes only bots with status IN ('active','paused')</t>
         </is>
       </c>
-      <c r="C7" s="100" t="inlineStr">
+      <c r="C7" s="107" t="inlineStr">
         <is>
           <t>1. D1 contains bots with various statuses including `active`, `paused`, `closed`, and `error`.</t>
         </is>
       </c>
-      <c r="D7" s="100" t="inlineStr">
+      <c r="D7" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit cron worker. 2. Observe which bots are read and processed.</t>
         </is>
       </c>
-      <c r="E7" s="100" t="inlineStr">
+      <c r="E7" s="107" t="inlineStr">
         <is>
           <t>1. Only bots with `bots.status IN ('active','paused')` are read from D1 and processed. Bots with `closed`, `error`, `idle`, or other statuses are excluded from the audit. (Reference: UC §2 Preconditions, FR-EXBOT-016, states.md row 71.)</t>
         </is>
       </c>
-      <c r="F7" s="100" t="inlineStr">
+      <c r="F7" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1" s="85">
-      <c r="A8" s="100" t="inlineStr">
+    <row r="8" ht="135" customHeight="1" s="85">
+      <c r="A8" s="107" t="inlineStr">
         <is>
           <t>TC_005</t>
         </is>
       </c>
-      <c r="B8" s="100" t="inlineStr">
+      <c r="B8" s="107" t="inlineStr">
         <is>
           <t>Verify reconcile mismatch triggers SAFE_MODE entry</t>
         </is>
       </c>
-      <c r="C8" s="100" t="inlineStr">
+      <c r="C8" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. The HL clearinghouseState returns an actual short size that differs from `hedge_legs.last_known_hl_short_size`.</t>
         </is>
       </c>
-      <c r="D8" s="100" t="inlineStr">
+      <c r="D8" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when the actual HL short size does not match the D1 recorded size.</t>
         </is>
       </c>
-      <c r="E8" s="100" t="inlineStr">
+      <c r="E8" s="107" t="inlineStr">
         <is>
           <t>1. Bot enters `safe_mode` (`bots.status='safe_mode'`). The mismatch is recorded in D1 with the size delta (actual minus expected). Admin notification is enqueued with message E-EXBOT-011: "Hedge position mismatch detected. Bot entered Safe Mode pending reconciliation." (Reference: AC-DA-02, FR-EXBOT-050, E-EXBOT-011.)</t>
         </is>
       </c>
-      <c r="F8" s="100" t="inlineStr">
+      <c r="F8" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="85">
-      <c r="A9" s="100" t="inlineStr">
+    <row r="9" ht="63" customHeight="1" s="85">
+      <c r="A9" s="107" t="inlineStr">
         <is>
           <t>TC_006</t>
         </is>
       </c>
-      <c r="B9" s="100" t="inlineStr">
+      <c r="B9" s="107" t="inlineStr">
         <is>
           <t>Verify reconcile mismatch records the size delta correctly when actual is greater</t>
         </is>
       </c>
-      <c r="C9" s="100" t="inlineStr">
+      <c r="C9" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. The actual HL short size is greater than `hedge_legs.last_known_hl_short_size`.</t>
         </is>
       </c>
-      <c r="D9" s="100" t="inlineStr">
+      <c r="D9" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker with a size mismatch where actual &gt; expected.</t>
         </is>
       </c>
-      <c r="E9" s="100" t="inlineStr">
+      <c r="E9" s="107" t="inlineStr">
         <is>
           <t>1. The D1 mismatch record stores the positive delta (actual minus expected). SAFE_MODE is triggered. (Reference: FR-EXBOT-050, UC A3.)</t>
         </is>
       </c>
-      <c r="F9" s="100" t="inlineStr">
+      <c r="F9" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" s="85">
-      <c r="A10" s="100" t="inlineStr">
+    <row r="10" ht="63" customHeight="1" s="85">
+      <c r="A10" s="107" t="inlineStr">
         <is>
           <t>TC_007</t>
         </is>
       </c>
-      <c r="B10" s="100" t="inlineStr">
+      <c r="B10" s="107" t="inlineStr">
         <is>
           <t>Verify reconcile mismatch records the size delta correctly when actual is less</t>
         </is>
       </c>
-      <c r="C10" s="100" t="inlineStr">
+      <c r="C10" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. The actual HL short size is less than `hedge_legs.last_known_hl_short_size`.</t>
         </is>
       </c>
-      <c r="D10" s="100" t="inlineStr">
+      <c r="D10" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker with a size mismatch where actual &lt; expected.</t>
         </is>
       </c>
-      <c r="E10" s="100" t="inlineStr">
+      <c r="E10" s="107" t="inlineStr">
         <is>
           <t>1. The D1 mismatch record stores the negative delta (actual minus expected). SAFE_MODE is triggered. (Reference: FR-EXBOT-050, UC A3.)</t>
         </is>
       </c>
-      <c r="F10" s="100" t="inlineStr">
+      <c r="F10" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1" s="85">
-      <c r="A11" s="100" t="inlineStr">
+    <row r="11" ht="123" customHeight="1" s="85">
+      <c r="A11" s="107" t="inlineStr">
         <is>
           <t>TC_008</t>
         </is>
       </c>
-      <c r="B11" s="100" t="inlineStr">
+      <c r="B11" s="107" t="inlineStr">
         <is>
           <t>Verify stop_trigger_crossed_at stuck for more than 30 minutes triggers SAFE_MODE</t>
         </is>
       </c>
-      <c r="C11" s="100" t="inlineStr">
+      <c r="C11" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_trigger_crossed_at` is set to a timestamp older than 30 minutes ago.</t>
         </is>
       </c>
-      <c r="D11" s="100" t="inlineStr">
+      <c r="D11" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when `stop_trigger_crossed_at` has been set for more than 30 minutes.</t>
         </is>
       </c>
-      <c r="E11" s="100" t="inlineStr">
+      <c r="E11" s="107" t="inlineStr">
         <is>
           <t>1. Bot enters `safe_mode` (`bots.status='safe_mode'`). Admin escalation notification is enqueued with message E-EXBOT-019: "Stop trigger marker stuck for over 30 minutes. Bot entered Safe Mode. Manual review required." (Reference: AC-DA-03, FR-EXBOT-033, FR-EXBOT-050, E-EXBOT-019.)</t>
         </is>
       </c>
-      <c r="F11" s="100" t="inlineStr">
+      <c r="F11" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1" s="85">
-      <c r="A12" s="100" t="inlineStr">
+    <row r="12" ht="87" customHeight="1" s="85">
+      <c r="A12" s="107" t="inlineStr">
         <is>
           <t>TC_009</t>
         </is>
       </c>
-      <c r="B12" s="100" t="inlineStr">
+      <c r="B12" s="107" t="inlineStr">
         <is>
           <t>Verify stuck detection boundary — age exactly 30 minutes does NOT trigger SAFE_MODE</t>
         </is>
       </c>
-      <c r="C12" s="100" t="inlineStr">
+      <c r="C12" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_trigger_crossed_at` is set to exactly 30 minutes ago.</t>
         </is>
       </c>
-      <c r="D12" s="100" t="inlineStr">
+      <c r="D12" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when the elapsed time since `stop_trigger_crossed_at` equals exactly 30 minutes.</t>
         </is>
       </c>
-      <c r="E12" s="100" t="inlineStr">
+      <c r="E12" s="107" t="inlineStr">
         <is>
           <t>1. The stuck condition evaluates to false (elapsed time is not greater than 30 minutes). No SAFE_MODE entry occurs. The audit proceeds to the next check. (Reference: FR-EXBOT-033, UC Step 4 boundary.)</t>
         </is>
       </c>
-      <c r="F12" s="100" t="inlineStr">
+      <c r="F12" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1" s="85">
-      <c r="A13" s="100" t="inlineStr">
+    <row r="13" ht="75" customHeight="1" s="85">
+      <c r="A13" s="107" t="inlineStr">
         <is>
           <t>TC_010</t>
         </is>
       </c>
-      <c r="B13" s="100" t="inlineStr">
+      <c r="B13" s="107" t="inlineStr">
         <is>
           <t>Verify stuck detection boundary — age exactly 31 minutes triggers SAFE_MODE</t>
         </is>
       </c>
-      <c r="C13" s="100" t="inlineStr">
+      <c r="C13" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_trigger_crossed_at` is set to exactly 31 minutes ago.</t>
         </is>
       </c>
-      <c r="D13" s="100" t="inlineStr">
+      <c r="D13" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when the elapsed time since `stop_trigger_crossed_at` is just over 30 minutes.</t>
         </is>
       </c>
-      <c r="E13" s="100" t="inlineStr">
+      <c r="E13" s="107" t="inlineStr">
         <is>
           <t>1. The stuck condition evaluates to true (31 minutes &gt; 30 minutes). SAFE_MODE is triggered with E-EXBOT-019. (Reference: FR-EXBOT-033, UC Step 4 boundary.)</t>
         </is>
       </c>
-      <c r="F13" s="100" t="inlineStr">
+      <c r="F13" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1" s="85">
-      <c r="A14" s="100" t="inlineStr">
+    <row r="14" ht="75" customHeight="1" s="85">
+      <c r="A14" s="107" t="inlineStr">
         <is>
           <t>TC_011</t>
         </is>
       </c>
-      <c r="B14" s="100" t="inlineStr">
+      <c r="B14" s="107" t="inlineStr">
         <is>
           <t>Verify stop_trigger_crossed_at being NULL skips the stuck check</t>
         </is>
       </c>
-      <c r="C14" s="100" t="inlineStr">
+      <c r="C14" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_trigger_crossed_at` is NULL.</t>
         </is>
       </c>
-      <c r="D14" s="100" t="inlineStr">
+      <c r="D14" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when `stop_trigger_crossed_at` is NULL.</t>
         </is>
       </c>
-      <c r="E14" s="100" t="inlineStr">
+      <c r="E14" s="107" t="inlineStr">
         <is>
           <t>1. The stuck condition evaluates to false (NULL fails the "IS NOT NULL" check). Worker proceeds to Step 5 without triggering SAFE_MODE. (Reference: BR-EXBOT-005, UC Step 4.)</t>
         </is>
       </c>
-      <c r="F14" s="100" t="inlineStr">
+      <c r="F14" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15.75" customHeight="1" s="85">
-      <c r="A15" s="100" t="inlineStr">
+    <row r="15" ht="123" customHeight="1" s="85">
+      <c r="A15" s="107" t="inlineStr">
         <is>
           <t>TC_012</t>
         </is>
       </c>
-      <c r="B15" s="100" t="inlineStr">
+      <c r="B15" s="107" t="inlineStr">
         <is>
           <t>Verify stop_replacing_started_at stuck for more than 60 seconds triggers SAFE_MODE</t>
         </is>
       </c>
-      <c r="C15" s="100" t="inlineStr">
+      <c r="C15" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_replacing_started_at` is set to a timestamp older than 60 seconds ago.</t>
         </is>
       </c>
-      <c r="D15" s="100" t="inlineStr">
+      <c r="D15" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when `stop_replacing_started_at` has been set for more than 60 seconds.</t>
         </is>
       </c>
-      <c r="E15" s="100" t="inlineStr">
+      <c r="E15" s="107" t="inlineStr">
         <is>
           <t>1. Bot enters `safe_mode` (`bots.status='safe_mode'`). Admin escalation notification is enqueued with message E-EXBOT-020: "Stop replacement marker stuck for over 60 seconds. Bot entered Safe Mode. Manual review required." (Reference: AC-DA-04, FR-EXBOT-033, FR-EXBOT-050, E-EXBOT-020.)</t>
         </is>
       </c>
-      <c r="F15" s="100" t="inlineStr">
+      <c r="F15" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1" s="85">
-      <c r="A16" s="100" t="inlineStr">
+    <row r="16" ht="87" customHeight="1" s="85">
+      <c r="A16" s="107" t="inlineStr">
         <is>
           <t>TC_013</t>
         </is>
       </c>
-      <c r="B16" s="100" t="inlineStr">
+      <c r="B16" s="107" t="inlineStr">
         <is>
           <t>Verify stuck detection boundary — age exactly 60 seconds does NOT trigger SAFE_MODE</t>
         </is>
       </c>
-      <c r="C16" s="100" t="inlineStr">
+      <c r="C16" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_replacing_started_at` is set to exactly 60 seconds ago.</t>
         </is>
       </c>
-      <c r="D16" s="100" t="inlineStr">
+      <c r="D16" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when the elapsed time since `stop_replacing_started_at` equals exactly 60 seconds.</t>
         </is>
       </c>
-      <c r="E16" s="100" t="inlineStr">
+      <c r="E16" s="107" t="inlineStr">
         <is>
           <t>1. The stuck condition evaluates to false (elapsed time is not greater than 60 seconds). No SAFE_MODE entry occurs. The audit proceeds to Step 6. (Reference: FR-EXBOT-033, UC Step 5 boundary.)</t>
         </is>
       </c>
-      <c r="F16" s="100" t="inlineStr">
+      <c r="F16" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="85">
-      <c r="A17" s="100" t="inlineStr">
+    <row r="17" ht="75" customHeight="1" s="85">
+      <c r="A17" s="107" t="inlineStr">
         <is>
           <t>TC_014</t>
         </is>
       </c>
-      <c r="B17" s="100" t="inlineStr">
+      <c r="B17" s="107" t="inlineStr">
         <is>
           <t>Verify stop_replacing_started_at being NULL skips the stuck check</t>
         </is>
       </c>
-      <c r="C17" s="100" t="inlineStr">
+      <c r="C17" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_replacing_started_at` is NULL.</t>
         </is>
       </c>
-      <c r="D17" s="100" t="inlineStr">
+      <c r="D17" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when `stop_replacing_started_at` is NULL.</t>
         </is>
       </c>
-      <c r="E17" s="100" t="inlineStr">
+      <c r="E17" s="107" t="inlineStr">
         <is>
           <t>1. The stuck condition evaluates to false (NULL fails the "IS NOT NULL" check). Worker proceeds to Step 6 without triggering SAFE_MODE. (Reference: FR-EXBOT-033, UC Step 5.)</t>
         </is>
       </c>
-      <c r="F17" s="100" t="inlineStr">
+      <c r="F17" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1" s="85">
-      <c r="A18" s="100" t="inlineStr">
+    <row r="18" ht="99" customHeight="1" s="85">
+      <c r="A18" s="107" t="inlineStr">
         <is>
           <t>TC_015</t>
         </is>
       </c>
-      <c r="B18" s="100" t="inlineStr">
+      <c r="B18" s="107" t="inlineStr">
         <is>
           <t>Verify deep-audit with zero active or paused bots completes without error</t>
         </is>
       </c>
-      <c r="C18" s="100" t="inlineStr">
+      <c r="C18" s="107" t="inlineStr">
         <is>
           <t>1. D1 contains no bots with `status IN ('active','paused')`.</t>
         </is>
       </c>
-      <c r="D18" s="100" t="inlineStr">
+      <c r="D18" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit cron worker when no qualifying bots exist.</t>
         </is>
       </c>
-      <c r="E18" s="100" t="inlineStr">
+      <c r="E18" s="107" t="inlineStr">
         <is>
           <t>1. The cron cycle completes successfully with no HL calls made, no D1 writes for bot records, and no notifications enqueued. The `queue_idempotency` row is still inserted for the audit cycle itself. (Reference: UC §2 Preconditions.)</t>
         </is>
       </c>
-      <c r="F18" s="100" t="inlineStr">
+      <c r="F18" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="85">
-      <c r="B19" s="99" t="inlineStr">
+    <row r="19" ht="39" customHeight="1" s="85">
+      <c r="A19" s="107" t="n"/>
+      <c r="B19" s="108" t="inlineStr">
         <is>
           <t>I.2. Integration &amp; State verification — Operation: Periodic Deep Audit (deep-audit)</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="85">
-      <c r="A20" s="100" t="inlineStr">
+      <c r="C19" s="107" t="n"/>
+      <c r="D19" s="107" t="n"/>
+      <c r="E19" s="107" t="n"/>
+      <c r="F19" s="107" t="n"/>
+    </row>
+    <row r="20" ht="135" customHeight="1" s="85">
+      <c r="A20" s="107" t="inlineStr">
         <is>
           <t>TC_016</t>
         </is>
       </c>
-      <c r="B20" s="100" t="inlineStr">
+      <c r="B20" s="107" t="inlineStr">
         <is>
           <t>Verify HL API unreachable causes graceful degradation without crashing the worker</t>
         </is>
       </c>
-      <c r="C20" s="100" t="inlineStr">
+      <c r="C20" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. HLRateLimitDO returns `{allowed: false}` or HL API returns a 5xx error.</t>
         </is>
       </c>
-      <c r="D20" s="100" t="inlineStr">
+      <c r="D20" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when the HL API is unreachable.</t>
         </is>
       </c>
-      <c r="E20" s="100" t="inlineStr">
+      <c r="E20" s="107" t="inlineStr">
         <is>
           <t>1. Steps 2, 3, 4, 6, and 7 (HL-dependent) are skipped. The cadence switches to the high-risk 1-hour interval. Notification "Hyperliquid API unreachable" with message E-EXBOT-008 is enqueued. Retry-pending state is recorded in D1. The bot stays in its current state. (Reference: AC-DA-05, UC A1, E-EXBOT-008.)</t>
         </is>
       </c>
-      <c r="F20" s="100" t="inlineStr">
+      <c r="F20" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="85">
-      <c r="A21" s="100" t="inlineStr">
+    <row r="21" ht="99" customHeight="1" s="85">
+      <c r="A21" s="107" t="inlineStr">
         <is>
           <t>TC_017</t>
         </is>
       </c>
-      <c r="B21" s="100" t="inlineStr">
+      <c r="B21" s="107" t="inlineStr">
         <is>
           <t>Verify deep-audit calls HL clearinghouseState with weight=2 via HLRateLimitDO</t>
         </is>
       </c>
-      <c r="C21" s="100" t="inlineStr">
+      <c r="C21" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. HLRateLimitDO has available weight budget (remaining weight &gt;= 2).</t>
         </is>
       </c>
-      <c r="D21" s="100" t="inlineStr">
+      <c r="D21" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker and observe the HL API call.</t>
         </is>
       </c>
-      <c r="E21" s="100" t="inlineStr">
+      <c r="E21" s="107" t="inlineStr">
         <is>
           <t>1. The worker calls HL clearinghouseState with declared weight=2 through HLRateLimitDO. BR-EXBOT-003 (HL weight=0) does NOT apply to deep-audit — this is the documented exception. (Reference: FR-EXBOT-091, UC Step 2.)</t>
         </is>
       </c>
-      <c r="F21" s="100" t="inlineStr">
+      <c r="F21" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1" s="85">
-      <c r="A22" s="100" t="inlineStr">
+    <row r="22" ht="75" customHeight="1" s="85">
+      <c r="A22" s="107" t="inlineStr">
         <is>
           <t>TC_018</t>
         </is>
       </c>
-      <c r="B22" s="100" t="inlineStr">
+      <c r="B22" s="107" t="inlineStr">
         <is>
           <t>Verify HLRateLimitDO returning false causes deep-audit to re-queue without proceeding</t>
         </is>
       </c>
-      <c r="C22" s="100" t="inlineStr">
+      <c r="C22" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. HLRateLimitDO has insufficient weight budget and returns `{allowed: false, retryAfterMs}`.</t>
         </is>
       </c>
-      <c r="D22" s="100" t="inlineStr">
+      <c r="D22" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when HLRateLimitDO denies the weight request.</t>
         </is>
       </c>
-      <c r="E22" s="100" t="inlineStr">
+      <c r="E22" s="107" t="inlineStr">
         <is>
           <t>1. The worker does NOT proceed with the HL call. The message is re-queued with the indicated delay. No partial state is written. (Reference: FR-EXBOT-091.)</t>
         </is>
       </c>
-      <c r="F22" s="100" t="inlineStr">
+      <c r="F22" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1" s="85">
-      <c r="A23" s="100" t="inlineStr">
+    <row r="23" ht="111" customHeight="1" s="85">
+      <c r="A23" s="107" t="inlineStr">
         <is>
           <t>TC_019</t>
         </is>
       </c>
-      <c r="B23" s="100" t="inlineStr">
+      <c r="B23" s="107" t="inlineStr">
         <is>
           <t>Verify partial HL failure — clearinghouseState succeeds but marginSummary fails</t>
         </is>
       </c>
-      <c r="C23" s="100" t="inlineStr">
+      <c r="C23" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. HL clearinghouseState call succeeds; HL marginSummary call fails with 5xx.</t>
         </is>
       </c>
-      <c r="D23" s="100" t="inlineStr">
+      <c r="D23" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker under partial HL failure (Step 2 succeeds, Step 6 fails).</t>
         </is>
       </c>
-      <c r="E23" s="100" t="inlineStr">
+      <c r="E23" s="107" t="inlineStr">
         <is>
           <t>1. Steps 2 and 3 complete normally. Step 6 (marginSummary) is skipped due to failure. Steps 7 and 8 (last_audit_at update, idempotency row) still complete. `hedge_legs.margin_status` retains its previous value (not updated). (Reference: UC Steps 2, 6, A1.)</t>
         </is>
       </c>
-      <c r="F23" s="100" t="inlineStr">
+      <c r="F23" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="85">
-      <c r="A24" s="100" t="inlineStr">
+    <row r="24" ht="111" customHeight="1" s="85">
+      <c r="A24" s="107" t="inlineStr">
         <is>
           <t>TC_020</t>
         </is>
       </c>
-      <c r="B24" s="100" t="inlineStr">
+      <c r="B24" s="107" t="inlineStr">
         <is>
           <t>Verify paused bot is fully audited including stuck marker detection</t>
         </is>
       </c>
-      <c r="C24" s="100" t="inlineStr">
+      <c r="C24" s="107" t="inlineStr">
         <is>
           <t>1. The bot has `bots.status='paused'` (lifecycle_state retained at pre-pause value). 2. No stuck markers are set. 3. HL API is reachable.</t>
         </is>
       </c>
-      <c r="D24" s="100" t="inlineStr">
+      <c r="D24" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit cron worker for the paused bot.</t>
         </is>
       </c>
-      <c r="E24" s="100" t="inlineStr">
+      <c r="E24" s="107" t="inlineStr">
         <is>
           <t>1. All detection paths (Steps 3–7) execute normally: clearinghouseState reconciliation, stuck marker checks, marginSummary fetch, and `last_audit_at` update. Pause does NOT skip deep-audit scheduling or any detection path. (Reference: AC-DA-06, FR-EXBOT-005, UC A2.)</t>
         </is>
       </c>
-      <c r="F24" s="100" t="inlineStr">
+      <c r="F24" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" s="85">
-      <c r="A25" s="100" t="inlineStr">
+    <row r="25" ht="87" customHeight="1" s="85">
+      <c r="A25" s="107" t="inlineStr">
         <is>
           <t>TC_021</t>
         </is>
       </c>
-      <c r="B25" s="100" t="inlineStr">
+      <c r="B25" s="107" t="inlineStr">
         <is>
           <t>Verify paused bot with stuck stop_trigger_crossed_at transitions paused to safe_mode</t>
         </is>
       </c>
-      <c r="C25" s="100" t="inlineStr">
+      <c r="C25" s="107" t="inlineStr">
         <is>
           <t>1. The bot has `bots.status='paused'` and `hedge_legs.stop_trigger_crossed_at` is set and aged more than 30 minutes.</t>
         </is>
       </c>
-      <c r="D25" s="100" t="inlineStr">
+      <c r="D25" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker for the paused bot with the stuck marker.</t>
         </is>
       </c>
-      <c r="E25" s="100" t="inlineStr">
+      <c r="E25" s="107" t="inlineStr">
         <is>
           <t>1. The bot transitions from `paused` to `safe_mode` (`bots.status='safe_mode'`). Admin escalation notification E-EXBOT-019 is enqueued. (Reference: FR-EXBOT-005, FR-EXBOT-033, FR-EXBOT-050, states.md row 71.)</t>
         </is>
       </c>
-      <c r="F25" s="100" t="inlineStr">
+      <c r="F25" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1" s="85">
-      <c r="A26" s="100" t="inlineStr">
+    <row r="26" ht="123" customHeight="1" s="85">
+      <c r="A26" s="107" t="inlineStr">
         <is>
           <t>TC_022</t>
         </is>
       </c>
-      <c r="B26" s="100" t="inlineStr">
+      <c r="B26" s="107" t="inlineStr">
         <is>
           <t>Verify both stuck markers set simultaneously — first condition triggers SAFE_MODE</t>
         </is>
       </c>
-      <c r="C26" s="100" t="inlineStr">
+      <c r="C26" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. Both `stop_trigger_crossed_at` (aged &gt;30 min) and `stop_replacing_started_at` (aged &gt;60s) are set simultaneously.</t>
         </is>
       </c>
-      <c r="D26" s="100" t="inlineStr">
+      <c r="D26" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when both stuck conditions are true.</t>
         </is>
       </c>
-      <c r="E26" s="100" t="inlineStr">
+      <c r="E26" s="107" t="inlineStr">
         <is>
           <t>1. Step 4 evaluates first — `stop_trigger_crossed_at` stuck is true. SAFE_MODE is triggered and E-EXBOT-019 is enqueued. Step 5 is not reached. Only E-EXBOT-019 notification is sent (first-triggered condition wins). (Reference: FR-EXBOT-033, FR-EXBOT-050, UC Steps 4–5 + A4.)</t>
         </is>
       </c>
-      <c r="F26" s="100" t="inlineStr">
+      <c r="F26" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="85">
-      <c r="A27" s="100" t="inlineStr">
+    <row r="27" ht="111" customHeight="1" s="85">
+      <c r="A27" s="107" t="inlineStr">
         <is>
           <t>TC_023</t>
         </is>
       </c>
-      <c r="B27" s="100" t="inlineStr">
+      <c r="B27" s="107" t="inlineStr">
         <is>
           <t>Verify circuit_breaker open triggers high-risk cadence switching to 1 hour</t>
         </is>
       </c>
-      <c r="C27" s="100" t="inlineStr">
+      <c r="C27" s="107" t="inlineStr">
         <is>
           <t>1. `circuit_breakers.state` is `open`. 2. The bot is in `active` status.</t>
         </is>
       </c>
-      <c r="D27" s="100" t="inlineStr">
+      <c r="D27" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when `circuit_breakers.state='open'`.</t>
         </is>
       </c>
-      <c r="E27" s="100" t="inlineStr">
+      <c r="E27" s="107" t="inlineStr">
         <is>
           <t>1. The cron schedule for this bot switches from the normal 6-hour interval to the high-risk 1-hour interval. Subsequent deep-audit runs occur every 1 hour until `circuit_breakers.state` returns to `closed`. (Reference: AC-DA-07, FR-EXBOT-040, UC §2 Preconditions.)</t>
         </is>
       </c>
-      <c r="F27" s="100" t="inlineStr">
+      <c r="F27" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1" s="85">
-      <c r="A28" s="100" t="inlineStr">
+    <row r="28" ht="87" customHeight="1" s="85">
+      <c r="A28" s="107" t="inlineStr">
         <is>
           <t>TC_024</t>
         </is>
       </c>
-      <c r="B28" s="100" t="inlineStr">
+      <c r="B28" s="107" t="inlineStr">
         <is>
           <t>Verify margin_status='warning' triggers high-risk cadence switching to 1 hour</t>
         </is>
       </c>
-      <c r="C28" s="100" t="inlineStr">
+      <c r="C28" s="107" t="inlineStr">
         <is>
           <t>1. The bot has `hedge_legs.margin_status='warning'`. 2. The bot is in `active` status.</t>
         </is>
       </c>
-      <c r="D28" s="100" t="inlineStr">
+      <c r="D28" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when `margin_status='warning'`.</t>
         </is>
       </c>
-      <c r="E28" s="100" t="inlineStr">
+      <c r="E28" s="107" t="inlineStr">
         <is>
           <t>1. The cron schedule switches from 6-hour to 1-hour interval. Note: if Step 6 updates `margin_status` from warning to ok, cadence may revert. (Reference: AC-DA-07, FR-EXBOT-060, UC §2 Preconditions.)</t>
         </is>
       </c>
-      <c r="F28" s="100" t="inlineStr">
+      <c r="F28" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1" s="85">
-      <c r="A29" s="100" t="inlineStr">
+    <row r="29" ht="51" customHeight="1" s="85">
+      <c r="A29" s="107" t="inlineStr">
         <is>
           <t>TC_025</t>
         </is>
       </c>
-      <c r="B29" s="100" t="inlineStr">
+      <c r="B29" s="107" t="inlineStr">
         <is>
           <t>Verify margin_status='critical' triggers high-risk cadence switching to 1 hour</t>
         </is>
       </c>
-      <c r="C29" s="100" t="inlineStr">
+      <c r="C29" s="107" t="inlineStr">
         <is>
           <t>1. The bot has `hedge_legs.margin_status='critical'`. 2. The bot is in `active` status.</t>
         </is>
       </c>
-      <c r="D29" s="100" t="inlineStr">
+      <c r="D29" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker when `margin_status='critical'`.</t>
         </is>
       </c>
-      <c r="E29" s="100" t="inlineStr">
+      <c r="E29" s="107" t="inlineStr">
         <is>
           <t>1. The cron schedule switches from 6-hour to 1-hour interval. (Reference: AC-DA-07, FR-EXBOT-060, UC §2 Preconditions.)</t>
         </is>
       </c>
-      <c r="F29" s="100" t="inlineStr">
+      <c r="F29" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="85">
-      <c r="A30" s="100" t="inlineStr">
+    <row r="30" ht="63" customHeight="1" s="85">
+      <c r="A30" s="107" t="inlineStr">
         <is>
           <t>TC_026</t>
         </is>
       </c>
-      <c r="B30" s="100" t="inlineStr">
+      <c r="B30" s="107" t="inlineStr">
         <is>
           <t>Verify normal 6-hour cadence is maintained when all conditions are nominal</t>
         </is>
       </c>
-      <c r="C30" s="100" t="inlineStr">
+      <c r="C30" s="107" t="inlineStr">
         <is>
           <t>1. The bot has `circuit_breakers.state='closed'` and `hedge_legs.margin_status='ok'`. 2. No stuck markers are set. 3. The bot is in `active` status.</t>
         </is>
       </c>
-      <c r="D30" s="100" t="inlineStr">
+      <c r="D30" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker under nominal conditions.</t>
         </is>
       </c>
-      <c r="E30" s="100" t="inlineStr">
+      <c r="E30" s="107" t="inlineStr">
         <is>
           <t>1. No cadence switching occurs. The deep-audit processes the bot at the normal 6-hour interval. (Reference: FR-EXBOT-016, UC §2 Preconditions.)</t>
         </is>
       </c>
-      <c r="F30" s="100" t="inlineStr">
+      <c r="F30" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="85">
-      <c r="A31" s="100" t="inlineStr">
+    <row r="31" ht="123" customHeight="1" s="85">
+      <c r="A31" s="107" t="inlineStr">
         <is>
           <t>TC_027</t>
         </is>
       </c>
-      <c r="B31" s="100" t="inlineStr">
+      <c r="B31" s="107" t="inlineStr">
         <is>
           <t>Verify queue idempotency — duplicate message delivery is rejected</t>
         </is>
       </c>
-      <c r="C31" s="100" t="inlineStr">
+      <c r="C31" s="107" t="inlineStr">
         <is>
           <t>1. A deep-audit message with a specific `message_id` has already been processed successfully (`queue_idempotency` row with `state='succeeded'`).</t>
         </is>
       </c>
-      <c r="D31" s="100" t="inlineStr">
+      <c r="D31" s="107" t="inlineStr">
         <is>
           <t>1. Re-deliver the same `message_id` in a new queue delivery.</t>
         </is>
       </c>
-      <c r="E31" s="100" t="inlineStr">
+      <c r="E31" s="107" t="inlineStr">
         <is>
           <t>1. The worker attempts to insert `queue_idempotency` with `state='started'` and hits a UNIQUE constraint conflict on `message_id`. The worker returns immediately without re-processing. The first delivery's `state='succeeded'` row remains intact. (Reference: AC-DA-08, FR-EXBOT-011.)</t>
         </is>
       </c>
-      <c r="F31" s="100" t="inlineStr">
+      <c r="F31" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1" s="85">
-      <c r="A32" s="100" t="inlineStr">
+    <row r="32" ht="87" customHeight="1" s="85">
+      <c r="A32" s="107" t="inlineStr">
         <is>
           <t>TC_028</t>
         </is>
       </c>
-      <c r="B32" s="100" t="inlineStr">
+      <c r="B32" s="107" t="inlineStr">
         <is>
           <t>Verify idempotency state progression — started to succeeded on first processing</t>
         </is>
       </c>
-      <c r="C32" s="100" t="inlineStr">
+      <c r="C32" s="107" t="inlineStr">
         <is>
           <t>1. A new deep-audit message with a unique `message_id` is received.</t>
         </is>
       </c>
-      <c r="D32" s="100" t="inlineStr">
+      <c r="D32" s="107" t="inlineStr">
         <is>
           <t>1. Process the new deep-audit message through to completion. 2. Read the `queue_idempotency` row state.</t>
         </is>
       </c>
-      <c r="E32" s="100" t="inlineStr">
+      <c r="E32" s="107" t="inlineStr">
         <is>
           <t>1. The worker inserts `queue_idempotency` with `state='started'` at the beginning. After successful completion, the row is updated to `state='succeeded'`. (Reference: FR-EXBOT-011, UC Step 8.)</t>
         </is>
       </c>
-      <c r="F32" s="100" t="inlineStr">
+      <c r="F32" s="107" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>High</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1" s="85">
-      <c r="A33" s="100" t="inlineStr">
+    <row r="33" ht="99" customHeight="1" s="85">
+      <c r="A33" s="107" t="inlineStr">
         <is>
           <t>TC_029</t>
         </is>
       </c>
-      <c r="B33" s="100" t="inlineStr">
+      <c r="B33" s="107" t="inlineStr">
         <is>
           <t>Verify deep-audit reads from correct D1 shard — bot state joined correctly</t>
         </is>
       </c>
-      <c r="C33" s="100" t="inlineStr">
+      <c r="C33" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status with valid records in `bots`, `hedge_legs`, and `circuit_breakers` tables (Phase A = 1 shard).</t>
         </is>
       </c>
-      <c r="D33" s="100" t="inlineStr">
+      <c r="D33" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker. 2. Observe the D1 reads: `bots.status`, `bots.lifecycle_state`, `hedge_legs`, `circuit_breakers.state`, `margin_status`.</t>
         </is>
       </c>
-      <c r="E33" s="100" t="inlineStr">
+      <c r="E33" s="107" t="inlineStr">
         <is>
           <t>1. Worker correctly joins `hedge_legs` to `bots` on `bot_id`. All fields are present and valid. Note: Phase B multi-shard iteration strategy is pending Tech Lead decision (Q-DA-03). (Reference: FR-EXBOT-016, NFR-EXBOT-012, UC Step 1.)</t>
         </is>
       </c>
-      <c r="F33" s="100" t="inlineStr">
+      <c r="F33" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1" s="85">
-      <c r="B34" s="99" t="inlineStr">
+    <row r="34" ht="39" customHeight="1" s="85">
+      <c r="A34" s="107" t="n"/>
+      <c r="B34" s="108" t="inlineStr">
         <is>
           <t>I.3. Non-functional (logic) verification — Operation: Periodic Deep Audit (deep-audit)</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1" s="85">
-      <c r="A35" s="100" t="inlineStr">
+      <c r="C34" s="107" t="n"/>
+      <c r="D34" s="107" t="n"/>
+      <c r="E34" s="107" t="n"/>
+      <c r="F34" s="107" t="n"/>
+    </row>
+    <row r="35" ht="123" customHeight="1" s="85">
+      <c r="A35" s="107" t="inlineStr">
         <is>
           <t>TC_030</t>
         </is>
       </c>
-      <c r="B35" s="100" t="inlineStr">
+      <c r="B35" s="107" t="inlineStr">
         <is>
           <t>Verify timestamp comparison for stuck detection uses precise arithmetic</t>
         </is>
       </c>
-      <c r="C35" s="100" t="inlineStr">
+      <c r="C35" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status. 2. `hedge_legs.stop_trigger_crossed_at` is set to a timestamp at the exact boundary of 30 minutes and 1 second ago.</t>
         </is>
       </c>
-      <c r="D35" s="100" t="inlineStr">
+      <c r="D35" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker and verify the stuck condition evaluation for `stop_trigger_crossed_at` and `stop_replacing_started_at`.</t>
         </is>
       </c>
-      <c r="E35" s="100" t="inlineStr">
+      <c r="E35" s="107" t="inlineStr">
         <is>
           <t>1. The timestamp arithmetic uses precise integer or BigDecimal comparison (not floating-point). Boundary cases (exactly 30 min / 60 sec) are evaluated correctly without rounding errors that could cause a false positive or false negative. (Reference: NFR-EXBOT-008, FR-EXBOT-033.)</t>
         </is>
       </c>
-      <c r="F35" s="100" t="inlineStr">
+      <c r="F35" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1" s="85">
-      <c r="A36" s="100" t="inlineStr">
+    <row r="36" ht="147" customHeight="1" s="85">
+      <c r="A36" s="107" t="inlineStr">
         <is>
           <t>TC_031</t>
         </is>
       </c>
-      <c r="B36" s="100" t="inlineStr">
+      <c r="B36" s="107" t="inlineStr">
         <is>
           <t>Verify deep-audit does not initiate bot_safe_close — SAFE_MODE is the extent of its role</t>
         </is>
       </c>
-      <c r="C36" s="100" t="inlineStr">
+      <c r="C36" s="107" t="inlineStr">
         <is>
           <t>1. The bot is in `active` status with a reconcile mismatch.</t>
         </is>
       </c>
-      <c r="D36" s="100" t="inlineStr">
+      <c r="D36" s="107" t="inlineStr">
         <is>
           <t>1. Trigger the deep-audit worker so it triggers SAFE_MODE entry.</t>
         </is>
       </c>
-      <c r="E36" s="100" t="inlineStr">
+      <c r="E36" s="107" t="inlineStr">
         <is>
           <t>1. Deep-audit triggers SAFE_MODE entry and enqueues admin notification. The worker does NOT initiate `bot_safe_close` — this is handled by the SAFE_MODE recovery logic per FR-EXBOT-050 and FR-EXBOT-072. The `close_operations` table is not affected by deep-audit alone. (Reference: UC §1.3 Out of Scope, FR-EXBOT-050, FR-EXBOT-072.)</t>
         </is>
       </c>
-      <c r="F36" s="100" t="inlineStr">
+      <c r="F36" s="107" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -26481,7 +26461,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>